<commit_message>
fixing broken tests after refactoring.
</commit_message>
<xml_diff>
--- a/Targets_V10p1.xlsx
+++ b/Targets_V10p1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/detector-simulator-py/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36B65B54-58B2-D04D-A4F8-A6B4036887F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADF42B1-0F04-5844-B33F-56C196D09E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2100" windowWidth="33600" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1960" windowWidth="33600" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>
@@ -465,7 +465,7 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>

</xml_diff>

<commit_message>
added excel import with mapping file
</commit_message>
<xml_diff>
--- a/Targets_V10p1.xlsx
+++ b/Targets_V10p1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/detector-simulator-py/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ADF42B1-0F04-5844-B33F-56C196D09E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF73521B-B94D-854A-9BEB-98CBE3827813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1960" windowWidth="33600" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="68800" yWindow="7800" windowWidth="33600" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
refactoring of required parameters. also added gaia lookup, but only stub for now
</commit_message>
<xml_diff>
--- a/Targets_V10p1.xlsx
+++ b/Targets_V10p1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/detector-simulator-py/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF73521B-B94D-854A-9BEB-98CBE3827813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B86CC3-23C6-A740-9D12-91CD41FE354E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="68800" yWindow="7800" windowWidth="33600" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -889,61 +889,13 @@
       <c r="U1" s="5"/>
     </row>
     <row r="2" spans="1:60" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="5" t="s">
         <v>19</v>
       </c>
       <c r="B2" t="s">
         <v>20</v>
       </c>
-      <c r="C2">
-        <v>2.7240329999999999</v>
-      </c>
-      <c r="D2">
-        <v>5.0529999999999999E-2</v>
-      </c>
-      <c r="E2">
-        <v>1.619</v>
-      </c>
-      <c r="F2">
-        <v>1.99</v>
-      </c>
-      <c r="G2">
-        <v>3353</v>
-      </c>
-      <c r="I2">
-        <v>8000</v>
-      </c>
-      <c r="J2">
-        <v>2.36</v>
-      </c>
-      <c r="K2">
-        <v>2.0299999999999998</v>
-      </c>
-      <c r="L2">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="M2">
-        <v>3.9</v>
-      </c>
-      <c r="N2">
-        <v>225.68673200000001</v>
-      </c>
-      <c r="O2">
-        <v>-3.0314874000000001</v>
-      </c>
-      <c r="P2">
-        <v>99.730999999999995</v>
-      </c>
-      <c r="Q2">
-        <v>6.5977600000000001</v>
-      </c>
-      <c r="R2">
-        <v>6.5536899999999996</v>
-      </c>
-      <c r="S2" s="3">
-        <f>(0.000000000000000138*G2/(1.673534E-24*1.3*0.000000066726*F2*1.8986E+30/(E2*7149200000)^2))/100000</f>
-        <v>1130.2166328238993</v>
-      </c>
+      <c r="S2" s="3"/>
       <c r="BE2" s="4"/>
       <c r="BG2" s="4"/>
       <c r="BH2" s="4"/>
@@ -1384,7 +1336,7 @@
       </c>
     </row>
     <row r="10" spans="1:60" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+      <c r="A10" s="5" t="s">
         <v>35</v>
       </c>
       <c r="B10" t="s">

</xml_diff>

<commit_message>
upload star classes, refactored excel readin and refactored tests. running green locally
</commit_message>
<xml_diff>
--- a/Targets_V10p1.xlsx
+++ b/Targets_V10p1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/detector-simulator-py/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B86CC3-23C6-A740-9D12-91CD41FE354E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE09A64B-918B-524D-998F-92679661DB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="68800" yWindow="7800" windowWidth="33600" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17940" yWindow="5140" windowWidth="33600" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>
@@ -889,13 +889,65 @@
       <c r="U1" s="5"/>
     </row>
     <row r="2" spans="1:60" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" t="s">
         <v>19</v>
       </c>
       <c r="B2" t="s">
         <v>20</v>
       </c>
-      <c r="S2" s="3"/>
+      <c r="C2">
+        <v>2.7240329999999999</v>
+      </c>
+      <c r="D2">
+        <v>5.0529999999999999E-2</v>
+      </c>
+      <c r="E2">
+        <v>1.619</v>
+      </c>
+      <c r="F2">
+        <v>1.99</v>
+      </c>
+      <c r="G2">
+        <v>3353</v>
+      </c>
+      <c r="I2">
+        <v>8000</v>
+      </c>
+      <c r="J2">
+        <v>2.36</v>
+      </c>
+      <c r="K2">
+        <v>2.0299999999999998</v>
+      </c>
+      <c r="L2">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="M2">
+        <v>3.9</v>
+      </c>
+      <c r="N2">
+        <v>225.68673200000001</v>
+      </c>
+      <c r="O2">
+        <v>-3.0314874000000001</v>
+      </c>
+      <c r="P2">
+        <v>99.730999999999995</v>
+      </c>
+      <c r="Q2">
+        <v>6.5977600000000001</v>
+      </c>
+      <c r="R2">
+        <v>6.5536899999999996</v>
+      </c>
+      <c r="S2" s="3">
+        <f>(0.000000000000000138*G2/(1.673534E-24*1.3*0.000000066726*F2*1.8986E+30/(E2*7149200000)^2))/100000</f>
+        <v>1130.2166328238993</v>
+      </c>
+      <c r="T2">
+        <f>IF(I2&gt;6800,-7,-5)</f>
+        <v>-7</v>
+      </c>
       <c r="BE2" s="4"/>
       <c r="BG2" s="4"/>
       <c r="BH2" s="4"/>
@@ -959,6 +1011,10 @@
         <f t="shared" ref="S3:S34" si="0">(0.000000000000000138*G3/(1.673534E-24*1.3*0.000000066726*F3*1.8986E+30/(E3*7149200000)^2))/100000</f>
         <v>1286.8653667451285</v>
       </c>
+      <c r="T3">
+        <f t="shared" ref="T3:T66" si="1">IF(I3&gt;6800,-7,-5)</f>
+        <v>-7</v>
+      </c>
       <c r="BE3" s="4"/>
       <c r="BG3" s="4"/>
       <c r="BH3" s="4"/>
@@ -1019,6 +1075,10 @@
         <f t="shared" si="0"/>
         <v>777.64358420307099</v>
       </c>
+      <c r="T4">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
       <c r="BE4" s="4"/>
       <c r="BG4" s="4"/>
       <c r="BH4" s="4"/>
@@ -1082,6 +1142,10 @@
         <f t="shared" si="0"/>
         <v>518.80488815900412</v>
       </c>
+      <c r="T5">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
       <c r="BE5" s="4"/>
       <c r="BG5" s="4"/>
       <c r="BH5" s="4"/>
@@ -1145,6 +1209,10 @@
         <f t="shared" si="0"/>
         <v>988.21070019970352</v>
       </c>
+      <c r="T6">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
       <c r="BE6" s="4"/>
       <c r="BG6" s="4"/>
       <c r="BH6" s="4"/>
@@ -1208,6 +1276,10 @@
         <f t="shared" si="0"/>
         <v>349.61677638948368</v>
       </c>
+      <c r="T7">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
       <c r="V7" s="2"/>
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
@@ -1271,6 +1343,10 @@
         <f t="shared" si="0"/>
         <v>797.33090232058362</v>
       </c>
+      <c r="T8">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
       <c r="V8" s="2"/>
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
@@ -1334,9 +1410,13 @@
         <f t="shared" si="0"/>
         <v>668.81110409377118</v>
       </c>
+      <c r="T9">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
     </row>
     <row r="10" spans="1:60" x14ac:dyDescent="0.2">
-      <c r="A10" s="5" t="s">
+      <c r="A10" t="s">
         <v>35</v>
       </c>
       <c r="B10" t="s">
@@ -1394,6 +1474,10 @@
         <f t="shared" si="0"/>
         <v>431.57254486096394</v>
       </c>
+      <c r="T10">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
     </row>
     <row r="11" spans="1:60" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -1454,6 +1538,10 @@
         <f t="shared" si="0"/>
         <v>3894.9775251994533</v>
       </c>
+      <c r="T11">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
       <c r="V11" s="2"/>
       <c r="Z11" s="2"/>
       <c r="AA11" s="2"/>
@@ -1517,6 +1605,10 @@
         <f t="shared" si="0"/>
         <v>211.51519610586323</v>
       </c>
+      <c r="T12">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
     </row>
     <row r="13" spans="1:60" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -1577,6 +1669,10 @@
         <f t="shared" si="0"/>
         <v>863.09804630713359</v>
       </c>
+      <c r="T13">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
     </row>
     <row r="14" spans="1:60" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
@@ -1637,6 +1733,10 @@
         <f t="shared" si="0"/>
         <v>599.63628364223177</v>
       </c>
+      <c r="T14">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
       <c r="V14" s="2"/>
       <c r="Z14" s="2"/>
       <c r="AA14" s="2"/>
@@ -1700,6 +1800,10 @@
         <f t="shared" si="0"/>
         <v>742.8583931109747</v>
       </c>
+      <c r="T15">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
     </row>
     <row r="16" spans="1:60" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -1760,11 +1864,15 @@
         <f t="shared" si="0"/>
         <v>789.006338593706</v>
       </c>
+      <c r="T16">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
       <c r="V16" s="2"/>
       <c r="Z16" s="2"/>
       <c r="AA16" s="2"/>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -1823,8 +1931,12 @@
         <f t="shared" si="0"/>
         <v>457.63140850776114</v>
       </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T17">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -1880,8 +1992,12 @@
         <f t="shared" si="0"/>
         <v>1280.5918535006856</v>
       </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T18">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>52</v>
       </c>
@@ -1940,8 +2056,12 @@
         <f t="shared" si="0"/>
         <v>99.730517672190274</v>
       </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T19">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>54</v>
       </c>
@@ -2000,8 +2120,12 @@
         <f t="shared" si="0"/>
         <v>574.11765847468712</v>
       </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T20">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>56</v>
       </c>
@@ -2060,8 +2184,12 @@
         <f t="shared" si="0"/>
         <v>965.25628287035329</v>
       </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T21">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>58</v>
       </c>
@@ -2120,8 +2248,12 @@
         <f t="shared" si="0"/>
         <v>570.64953846380126</v>
       </c>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T22">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>59</v>
       </c>
@@ -2180,8 +2312,12 @@
         <f t="shared" si="0"/>
         <v>39.515068300859213</v>
       </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T23">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>60</v>
       </c>
@@ -2240,8 +2376,12 @@
         <f t="shared" si="0"/>
         <v>597.79498778467087</v>
       </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T24">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>61</v>
       </c>
@@ -2300,8 +2440,12 @@
         <f t="shared" si="0"/>
         <v>974.78820571370204</v>
       </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T25">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>63</v>
       </c>
@@ -2360,8 +2504,12 @@
         <f t="shared" si="0"/>
         <v>795.95548671567838</v>
       </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T26">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>65</v>
       </c>
@@ -2417,8 +2565,12 @@
         <f t="shared" si="0"/>
         <v>77.040187113891676</v>
       </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T27">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>66</v>
       </c>
@@ -2477,8 +2629,12 @@
         <f t="shared" si="0"/>
         <v>267.77715667890726</v>
       </c>
-    </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T28">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>68</v>
       </c>
@@ -2537,8 +2693,12 @@
         <f t="shared" si="0"/>
         <v>948.15286253702118</v>
       </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T29">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>69</v>
       </c>
@@ -2597,8 +2757,12 @@
         <f t="shared" si="0"/>
         <v>36.149567272802649</v>
       </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T30">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>70</v>
       </c>
@@ -2657,8 +2821,12 @@
         <f t="shared" si="0"/>
         <v>882.20971786077962</v>
       </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T31">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>72</v>
       </c>
@@ -2717,8 +2885,12 @@
         <f t="shared" si="0"/>
         <v>93.704022194109143</v>
       </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T32">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>74</v>
       </c>
@@ -2777,8 +2949,12 @@
         <f t="shared" si="0"/>
         <v>1277.1766379712274</v>
       </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T33">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>76</v>
       </c>
@@ -2837,8 +3013,12 @@
         <f t="shared" si="0"/>
         <v>1103.5971886171305</v>
       </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T34">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>77</v>
       </c>
@@ -2894,11 +3074,15 @@
         <v>9.20974</v>
       </c>
       <c r="S35">
-        <f t="shared" ref="S35:S66" si="1">(0.000000000000000138*G35/(1.673534E-24*1.3*0.000000066726*F35*1.8986E+30/(E35*7149200000)^2))/100000</f>
+        <f t="shared" ref="S35:S66" si="2">(0.000000000000000138*G35/(1.673534E-24*1.3*0.000000066726*F35*1.8986E+30/(E35*7149200000)^2))/100000</f>
         <v>140.68549179703928</v>
       </c>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T35">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>78</v>
       </c>
@@ -2951,11 +3135,15 @@
         <v>9.3503900000000009</v>
       </c>
       <c r="S36">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>353.31388599481477</v>
       </c>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T36">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>79</v>
       </c>
@@ -3008,11 +3196,15 @@
         <v>9.4517399999999991</v>
       </c>
       <c r="S37">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>338.15838787809196</v>
       </c>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T37">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>80</v>
       </c>
@@ -3068,11 +3260,15 @@
         <v>9.3251000000000008</v>
       </c>
       <c r="S38">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>162.15983922320817</v>
       </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T38">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>81</v>
       </c>
@@ -3128,11 +3324,15 @@
         <v>9.4290710000000004</v>
       </c>
       <c r="S39">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>56.120615203365361</v>
       </c>
-    </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T39">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>82</v>
       </c>
@@ -3185,11 +3385,15 @@
         <v>9.3767099999999992</v>
       </c>
       <c r="S40">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>701.18164217622461</v>
       </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T40">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>83</v>
       </c>
@@ -3245,11 +3449,15 @@
         <v>9.3950700000000005</v>
       </c>
       <c r="S41">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2192.2225820487197</v>
       </c>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T41">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>84</v>
       </c>
@@ -3302,11 +3510,15 @@
         <v>9.3678899999999992</v>
       </c>
       <c r="S42">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1399.2265914107247</v>
       </c>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T42">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>85</v>
       </c>
@@ -3362,11 +3574,15 @@
         <v>9.4135299999999997</v>
       </c>
       <c r="S43">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1175.9460676296278</v>
       </c>
-    </row>
-    <row r="44" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T43">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>86</v>
       </c>
@@ -3419,11 +3635,15 @@
         <v>9.4724400000000006</v>
       </c>
       <c r="S44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>83.670803141549356</v>
       </c>
-    </row>
-    <row r="45" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T44">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>87</v>
       </c>
@@ -3476,11 +3696,15 @@
         <v>9.5202500000000008</v>
       </c>
       <c r="S45">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>934.76971602454307</v>
       </c>
-    </row>
-    <row r="46" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T45">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>88</v>
       </c>
@@ -3536,11 +3760,15 @@
         <v>9.5843900000000009</v>
       </c>
       <c r="S46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1460.8182255852041</v>
       </c>
-    </row>
-    <row r="47" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T46">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>89</v>
       </c>
@@ -3593,11 +3821,15 @@
         <v>9.5635499999999993</v>
       </c>
       <c r="S47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2101.5864855136347</v>
       </c>
-    </row>
-    <row r="48" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T47">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>90</v>
       </c>
@@ -3650,11 +3882,15 @@
         <v>9.6464700000000008</v>
       </c>
       <c r="S48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>103.20465157174387</v>
       </c>
-    </row>
-    <row r="49" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T48">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>91</v>
       </c>
@@ -3710,11 +3946,15 @@
         <v>9.5723000000000003</v>
       </c>
       <c r="S49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1226.0598654781754</v>
       </c>
-    </row>
-    <row r="50" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T49">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>93</v>
       </c>
@@ -3767,11 +4007,15 @@
         <v>9.6080000000000005</v>
       </c>
       <c r="S50">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1039.84328949877</v>
       </c>
-    </row>
-    <row r="51" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T50">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>94</v>
       </c>
@@ -3827,11 +4071,15 @@
         <v>9.5193600000000007</v>
       </c>
       <c r="S51">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>200.46131426194896</v>
       </c>
-    </row>
-    <row r="52" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T51">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>96</v>
       </c>
@@ -3884,11 +4132,15 @@
         <v>9.77332</v>
       </c>
       <c r="S52">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>387.53401759458865</v>
       </c>
-    </row>
-    <row r="53" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T52">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>97</v>
       </c>
@@ -3944,11 +4196,15 @@
         <v>9.6124899999999993</v>
       </c>
       <c r="S53">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>136.24063220140397</v>
       </c>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T53">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>99</v>
       </c>
@@ -4004,11 +4260,15 @@
         <v>9.6000599999999991</v>
       </c>
       <c r="S54">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>972.96006983022733</v>
       </c>
-    </row>
-    <row r="55" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T54">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>101</v>
       </c>
@@ -4061,11 +4321,15 @@
         <v>10.367800000000001</v>
       </c>
       <c r="S55">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>160.76196513632402</v>
       </c>
-    </row>
-    <row r="56" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T55">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>102</v>
       </c>
@@ -4121,11 +4385,15 @@
         <v>9.6495599999999992</v>
       </c>
       <c r="S56">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>956.09264119622901</v>
       </c>
-    </row>
-    <row r="57" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T56">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>103</v>
       </c>
@@ -4178,11 +4446,15 @@
         <v>9.6598100000000002</v>
       </c>
       <c r="S57">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1324.5165539963698</v>
       </c>
-    </row>
-    <row r="58" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T57">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>104</v>
       </c>
@@ -4235,11 +4507,15 @@
         <v>9.7632399999999997</v>
       </c>
       <c r="S58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>582.97620763372299</v>
       </c>
-    </row>
-    <row r="59" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T58">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>105</v>
       </c>
@@ -4292,11 +4568,15 @@
         <v>9.7262599999999999</v>
       </c>
       <c r="S59">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>662.28004924519439</v>
       </c>
-    </row>
-    <row r="60" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T59">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>106</v>
       </c>
@@ -4352,11 +4632,15 @@
         <v>9.6608199999999993</v>
       </c>
       <c r="S60">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>355.42536038318485</v>
       </c>
-    </row>
-    <row r="61" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T60">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>107</v>
       </c>
@@ -4412,11 +4696,15 @@
         <v>10.178599999999999</v>
       </c>
       <c r="S61">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1121.1126749906216</v>
       </c>
-    </row>
-    <row r="62" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T61">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>108</v>
       </c>
@@ -4472,11 +4760,15 @@
         <v>9.7388899999999996</v>
       </c>
       <c r="S62">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>120.66830436099001</v>
       </c>
-    </row>
-    <row r="63" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T62">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>110</v>
       </c>
@@ -4532,11 +4824,15 @@
         <v>9.8633100000000002</v>
       </c>
       <c r="S63">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>443.85469120292152</v>
       </c>
-    </row>
-    <row r="64" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T63">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>112</v>
       </c>
@@ -4589,11 +4885,15 @@
         <v>9.7596699999999998</v>
       </c>
       <c r="S64">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>55.915145726222889</v>
       </c>
-    </row>
-    <row r="65" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T64">
+        <f t="shared" si="1"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>113</v>
       </c>
@@ -4649,11 +4949,15 @@
         <v>9.4846599999999999</v>
       </c>
       <c r="S65">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>955.72600175951948</v>
       </c>
-    </row>
-    <row r="66" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T65">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>115</v>
       </c>
@@ -4706,11 +5010,15 @@
         <v>9.7295700000000007</v>
       </c>
       <c r="S66">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>487.59044264912109</v>
       </c>
-    </row>
-    <row r="67" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T66">
+        <f t="shared" si="1"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>116</v>
       </c>
@@ -4766,11 +5074,15 @@
         <v>9.7777600000000007</v>
       </c>
       <c r="S67">
-        <f t="shared" ref="S67:S79" si="2">(0.000000000000000138*G67/(1.673534E-24*1.3*0.000000066726*F67*1.8986E+30/(E67*7149200000)^2))/100000</f>
+        <f t="shared" ref="S67:S79" si="3">(0.000000000000000138*G67/(1.673534E-24*1.3*0.000000066726*F67*1.8986E+30/(E67*7149200000)^2))/100000</f>
         <v>755.33252275944176</v>
       </c>
-    </row>
-    <row r="68" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T67">
+        <f t="shared" ref="T67:T79" si="4">IF(I67&gt;6800,-7,-5)</f>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>118</v>
       </c>
@@ -4826,11 +5138,15 @@
         <v>9.9122599999999998</v>
       </c>
       <c r="S68">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1247.4798366438731</v>
       </c>
-    </row>
-    <row r="69" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T68">
+        <f t="shared" si="4"/>
+        <v>-7</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>120</v>
       </c>
@@ -4886,11 +5202,15 @@
         <v>9.8465900000000008</v>
       </c>
       <c r="S69">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>224.58825733889913</v>
       </c>
-    </row>
-    <row r="70" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T69">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>122</v>
       </c>
@@ -4943,11 +5263,15 @@
         <v>9.641</v>
       </c>
       <c r="S70">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>318.17832033985127</v>
       </c>
-    </row>
-    <row r="71" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T70">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>123</v>
       </c>
@@ -5003,11 +5327,15 @@
         <v>9.8192900000000005</v>
       </c>
       <c r="S71">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>621.55661806820979</v>
       </c>
-    </row>
-    <row r="72" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T71">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>124</v>
       </c>
@@ -5063,11 +5391,15 @@
         <v>9.95702</v>
       </c>
       <c r="S72">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1492.9814393090719</v>
       </c>
-    </row>
-    <row r="73" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T72">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="73" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>125</v>
       </c>
@@ -5123,11 +5455,15 @@
         <v>9.8728300000000004</v>
       </c>
       <c r="S73">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>243.60813720463176</v>
       </c>
-    </row>
-    <row r="74" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T73">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>127</v>
       </c>
@@ -5183,11 +5519,15 @@
         <v>9.9720200000000006</v>
       </c>
       <c r="S74">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1209.5375438309629</v>
       </c>
-    </row>
-    <row r="75" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T74">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="75" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>129</v>
       </c>
@@ -5243,11 +5583,15 @@
         <v>10.028499999999999</v>
       </c>
       <c r="S75">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2049.4439875099679</v>
       </c>
-    </row>
-    <row r="76" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T75">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="76" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>130</v>
       </c>
@@ -5303,11 +5647,15 @@
         <v>9.9823299999999993</v>
       </c>
       <c r="S76">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1107.9861243219782</v>
       </c>
-    </row>
-    <row r="77" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T76">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="77" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>132</v>
       </c>
@@ -5363,11 +5711,15 @@
         <v>9.8670799999999996</v>
       </c>
       <c r="S77">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2057.1154637812851</v>
       </c>
-    </row>
-    <row r="78" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T77">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>133</v>
       </c>
@@ -5423,11 +5775,15 @@
         <v>9.8979599999999994</v>
       </c>
       <c r="S78">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1257.117296864338</v>
       </c>
-    </row>
-    <row r="79" spans="1:19" x14ac:dyDescent="0.2">
+      <c r="T78">
+        <f t="shared" si="4"/>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>134</v>
       </c>
@@ -5483,8 +5839,12 @@
         <v>9.9369700000000005</v>
       </c>
       <c r="S79">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>422.11900227636102</v>
+      </c>
+      <c r="T79">
+        <f t="shared" si="4"/>
+        <v>-5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
removed old functions and added new tests
</commit_message>
<xml_diff>
--- a/Targets_V10p1.xlsx
+++ b/Targets_V10p1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/andreatanzer/Documents/Space Science/MasterThesis/detector-simulator-py/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE09A64B-918B-524D-998F-92679661DB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49627D60-0368-7E4C-ABB6-9824CB6B704C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17940" yWindow="5140" windowWidth="33600" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22580" yWindow="2300" windowWidth="33600" windowHeight="17400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Targets_V10p1" sheetId="1" r:id="rId1"/>

</xml_diff>